<commit_message>
Implemented team member names
</commit_message>
<xml_diff>
--- a/Homework 04 - Risk Register and Comm Plan.xlsx
+++ b/Homework 04 - Risk Register and Comm Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9c7c63b8d3e1e1c/School/4 - Info Sys Proj Mgmt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="343" documentId="11_F25DC773A252ABDACC1048EEF9187A645BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0700455-5901-466C-BE4C-DCEFAB29AF66}"/>
+  <xr:revisionPtr revIDLastSave="387" documentId="11_F25DC773A252ABDACC1048EEF9187A645BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0016484F-05A7-46D5-9040-534D001DEB82}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Risk Identification" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="127">
   <si>
     <t>Category</t>
   </si>
@@ -47,9 +47,6 @@
     <t>Technical</t>
   </si>
   <si>
-    <t>Techincal</t>
-  </si>
-  <si>
     <t>Third-party mapping/navigation API failure</t>
   </si>
   <si>
@@ -227,24 +224,6 @@
     <t>R-16</t>
   </si>
   <si>
-    <t>Mapping &amp; Location Services Team</t>
-  </si>
-  <si>
-    <t>Payment Integration Team</t>
-  </si>
-  <si>
-    <t>Backend/API Team</t>
-  </si>
-  <si>
-    <t>Project Manager</t>
-  </si>
-  <si>
-    <t>QA &amp; Testing Team</t>
-  </si>
-  <si>
-    <t>Development Team Leads</t>
-  </si>
-  <si>
     <t>Mitigate</t>
   </si>
   <si>
@@ -332,9 +311,6 @@
     <t>Project Closure Meeting</t>
   </si>
   <si>
-    <t>Twice a week</t>
-  </si>
-  <si>
     <t>Beginning of each sprint</t>
   </si>
   <si>
@@ -365,27 +341,6 @@
     <t>Teams / Email</t>
   </si>
   <si>
-    <t>Development Teams &amp; Team Leads</t>
-  </si>
-  <si>
-    <t>Project Manager, Team Leads &amp; Development Teams</t>
-  </si>
-  <si>
-    <t>Project Manager &amp; Stakeholders</t>
-  </si>
-  <si>
-    <t>Project Team &amp; Stakeholders</t>
-  </si>
-  <si>
-    <t>Project Manager &amp; Team Leads</t>
-  </si>
-  <si>
-    <t>Project Manager, Risk Owner &amp; Affected Team Leads</t>
-  </si>
-  <si>
-    <t>Project Team &amp; Key Stakeholders</t>
-  </si>
-  <si>
     <t>Share progress, identify blockers, and coordinate current development tasks.</t>
   </si>
   <si>
@@ -405,6 +360,54 @@
   </si>
   <si>
     <t>Review final deliverables, obtain approval, document lessons learned, and formally close the project.</t>
+  </si>
+  <si>
+    <t>William Cooke</t>
+  </si>
+  <si>
+    <t>Charles Byrne</t>
+  </si>
+  <si>
+    <t>Chalres Byrne</t>
+  </si>
+  <si>
+    <t>Ayden Moss</t>
+  </si>
+  <si>
+    <t>Alex Rivera</t>
+  </si>
+  <si>
+    <t>Paige Hoffman</t>
+  </si>
+  <si>
+    <t>The Risk Register has been updated to assign ownership to specific project team members based on the roles established in the Resource Plan. Technical and integration risks are assigned to the appropriate specialists, while broader scheduling, staffing, and stakeholder risks remain under the Project Manager. These assignments improve accountability and establish clear responsibility for monitoring and responding to risks throughout the project.</t>
+  </si>
+  <si>
+    <t>All eight project team members</t>
+  </si>
+  <si>
+    <t>Project team and stakeholders</t>
+  </si>
+  <si>
+    <t>Alex Rivera, Charles Byrne, and the development team</t>
+  </si>
+  <si>
+    <t>Alex Rivera --&gt; Project Stakeholders</t>
+  </si>
+  <si>
+    <t>Alex Rivera and relevant risk owners</t>
+  </si>
+  <si>
+    <t>Alex Rivera, risk owner, affected team members</t>
+  </si>
+  <si>
+    <t>All eight team members and key stakeholders</t>
+  </si>
+  <si>
+    <t>Twice weekly</t>
+  </si>
+  <si>
+    <t>The Communication Plan has been refined to align with the finalized project staffing structure and Risk Register. Meeting participants and reporting responsibilities now reflect the established project roles, with risk owners involved in relevant reviews and escalations. The existing meeting schedule and communication methods remain unchanged, as they continue to support the project's planned development activities.</t>
   </si>
 </sst>
 </file>
@@ -491,31 +494,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -687,6 +691,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5C29398B-FFDC-46EE-8C10-4C06357E1A4B}" name="Table1" displayName="Table1" ref="A1:E17" totalsRowShown="0">
   <autoFilter ref="A1:E17" xr:uid="{5C29398B-FFDC-46EE-8C10-4C06357E1A4B}"/>
@@ -718,14 +726,14 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1462BB64-0A56-4336-814C-CB003290076A}" name="Table3" displayName="Table3" ref="A1:E8" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1462BB64-0A56-4336-814C-CB003290076A}" name="Table3" displayName="Table3" ref="A1:E8" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <autoFilter ref="A1:E8" xr:uid="{1462BB64-0A56-4336-814C-CB003290076A}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{A55B4FEE-100F-4BD0-9154-40C2A87E262F}" name="Meeting/Report" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{1BBAAC29-6A63-47FE-AE0B-5A89899F1BCB}" name="Cadence" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{3E3F9B8D-2C7A-4220-AC89-B4D9BF2D9762}" name="Method" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{809C358E-F3E3-49C3-8927-7842BAD57478}" name="Participants" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{2068F1D7-CA8F-43A9-8FF4-A072572B1F7F}" name="Purpose/Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{A55B4FEE-100F-4BD0-9154-40C2A87E262F}" name="Meeting/Report" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{1BBAAC29-6A63-47FE-AE0B-5A89899F1BCB}" name="Cadence" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{3E3F9B8D-2C7A-4220-AC89-B4D9BF2D9762}" name="Method" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{809C358E-F3E3-49C3-8927-7842BAD57478}" name="Participants" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{2068F1D7-CA8F-43A9-8FF4-A072572B1F7F}" name="Purpose/Notes" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1024,272 +1032,272 @@
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="C4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>22</v>
+        <v>14</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" t="s">
         <v>15</v>
       </c>
-      <c r="D9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>25</v>
+      <c r="E9" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="C10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C11" t="s">
-        <v>35</v>
-      </c>
-      <c r="D11" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="C12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D12" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="C13" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" t="s">
-        <v>15</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D14" t="s">
-        <v>16</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>41</v>
+        <v>15</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="C15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" t="s">
         <v>15</v>
       </c>
-      <c r="D15" t="s">
-        <v>16</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>42</v>
+      <c r="E15" s="1" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>38</v>
       </c>
       <c r="C16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D16" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>43</v>
+        <v>14</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>40</v>
+        <v>35</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="C17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>15</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>44</v>
+        <v>14</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1302,7 +1310,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0FA6544-68EE-4732-AD7B-A0D356731EFE}">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" customWidth="1"/>
@@ -1314,397 +1322,411 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C1" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="G1" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="G1" s="8" t="s">
+    </row>
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="7" t="s">
+      <c r="B2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" s="10" t="s">
         <v>66</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="G2" s="11" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="B4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G4" s="10" t="s">
         <v>68</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>113</v>
+      </c>
+      <c r="F5" t="s">
+        <v>65</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" t="s">
-        <v>68</v>
-      </c>
-      <c r="F5" t="s">
-        <v>72</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>77</v>
+      <c r="B6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" t="s">
+        <v>114</v>
+      </c>
+      <c r="F7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" t="s">
-        <v>70</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="C8" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G8" s="10" t="s">
         <v>72</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" t="s">
+        <v>115</v>
+      </c>
+      <c r="F9" t="s">
+        <v>65</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" t="s">
-        <v>69</v>
-      </c>
-      <c r="F9" t="s">
-        <v>72</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>81</v>
+      <c r="B10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" t="s">
+        <v>116</v>
+      </c>
+      <c r="F11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B11" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" t="s">
-        <v>68</v>
-      </c>
-      <c r="F11" t="s">
-        <v>72</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>83</v>
+      <c r="B12" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" t="s">
+        <v>115</v>
+      </c>
+      <c r="F13" t="s">
+        <v>65</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B13" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="12" t="s">
+      <c r="B14" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E13" t="s">
-        <v>69</v>
-      </c>
-      <c r="F13" t="s">
-        <v>72</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>85</v>
+      <c r="E14" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" t="s">
+        <v>115</v>
+      </c>
+      <c r="F15" t="s">
+        <v>65</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B16" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="E15" t="s">
-        <v>69</v>
-      </c>
-      <c r="F15" t="s">
-        <v>72</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>87</v>
+      <c r="C16" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" t="s">
+        <v>115</v>
+      </c>
+      <c r="F17" t="s">
         <v>65</v>
       </c>
-      <c r="B17" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="E17" t="s">
-        <v>69</v>
-      </c>
-      <c r="F17" t="s">
-        <v>72</v>
-      </c>
-      <c r="G17" s="10" t="s">
-        <v>88</v>
-      </c>
+      <c r="G17" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A19:G19"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1715,7 +1737,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EABBC31B-8A6E-4966-9FBC-AA6D5B595462}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="28.5703125" customWidth="1"/>
@@ -1724,142 +1746,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B4" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="B5" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="B6" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="B7" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="C8" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>125</v>
-      </c>
+    </row>
+    <row r="10" spans="1:5" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A10:E10"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>